<commit_message>
Updated ESP_grids_kan model - 2026-04-29 18:52
</commit_message>
<xml_diff>
--- a/VerveStacks_ESP_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ESP_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ESP_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{857D1FFB-1CF4-4E8D-AB75-52860D725BE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B38774EE-15B7-4E80-A3A2-9F3413EB4695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5086,7 +5086,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E38F60B0-DD02-4D52-ACE7-031EE006A7C9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14B84472-B842-403D-8034-935E2EBC2E36}">
   <dimension ref="B9:H355"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -34626,7 +34626,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFF71613-490A-46B5-B019-83908D15BD18}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37B15722-3BF8-4DE6-B071-29CC1663D534}">
   <dimension ref="B9:L355"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>